<commit_message>
Fix flow accounting, preserve guest drafts and validate complete release
</commit_message>
<xml_diff>
--- a/docs/submission/current/sample-report.xlsx
+++ b/docs/submission/current/sample-report.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2585" uniqueCount="989">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2600" uniqueCount="997">
   <si>
     <t>Предварительная оценка роботизации</t>
   </si>
@@ -31,7 +31,7 @@
     <t>Проект</t>
   </si>
   <si>
-    <t>Сдаточный пример - полный цикл стеллажа N6 C2</t>
+    <t>Сдаточный пример - полный цикл мобильного стеллажа</t>
   </si>
   <si>
     <t>Тип объекта</t>
@@ -43,25 +43,25 @@
     <t>Дата расчёта</t>
   </si>
   <si>
-    <t>18.10.2026 16:04 МСК</t>
+    <t>18.10.2026 17:35 МСК</t>
   </si>
   <si>
     <t>Модель расчёта</t>
   </si>
   <si>
-    <t>tz-1.0.5</t>
+    <t>tz-1.0.6</t>
   </si>
   <si>
     <t>Модель имитации</t>
   </si>
   <si>
-    <t>sim-1.1.0</t>
+    <t>sim-1.2.0</t>
   </si>
   <si>
     <t>Версия данных</t>
   </si>
   <si>
-    <t>744ad95b</t>
+    <t>f4935a60</t>
   </si>
   <si>
     <t>Вывод</t>
@@ -169,7 +169,7 @@
     <t>Имитация</t>
   </si>
   <si>
-    <t>Проверка 3D текущего входа: OK; Заданные критерии модели выполнены; фактический результат пилота не проверен.; 52 из 52 ед./ч; очередь 2; модель warehouse-dense-underlift-1.7.2</t>
+    <t>Проверка 3D текущего входа: OK; Заданные критерии модели выполнены; фактический результат пилота не проверен.; 52 из 52 ед./ч; очередь 2; модель warehouse-dense-underlift-1.8.0</t>
   </si>
   <si>
     <t>Риски</t>
@@ -1906,6 +1906,15 @@
     <t>Расчёт подтверждён имитацией</t>
   </si>
   <si>
+    <t>Наблюдалось клиентских заданий в пике</t>
+  </si>
+  <si>
+    <t>Состав потока: приёмка / отгрузка / внутренние</t>
+  </si>
+  <si>
+    <t>50 / 50 / 0 %</t>
+  </si>
+  <si>
     <t>Роботов в прогоне</t>
   </si>
   <si>
@@ -1936,7 +1945,7 @@
     <t>Зерно генератора</t>
   </si>
   <si>
-    <t>warehouse-dense-underlift-1.7.2</t>
+    <t>warehouse-dense-underlift-1.8.0</t>
   </si>
   <si>
     <t>Группа</t>
@@ -2383,6 +2392,15 @@
     <t>Если даже в пик роботы простаивают 40 % времени и больше, парк избыточен и его стоит уменьшить. Порог — наша оценка; вместе с перебором минимального парка он показывает запас.</t>
   </si>
   <si>
+    <t>Начальная доля свободных мест для внутренних перемещений</t>
+  </si>
+  <si>
+    <t>simStorageVacancyShare</t>
+  </si>
+  <si>
+    <t>Явное модельное допущение, не измерение склада и не типовой норматив: при внутренних перемещениях эта доля существующих мест изначально свободна. Число округляется вниз. Полный склад без свободных мест не подтверждает перенос стеллажа на новое место. При отсутствии внутренних перемещений состав носителей не меняется.</t>
+  </si>
+  <si>
     <t>Прогрев имитации на среднем потоке</t>
   </si>
   <si>
@@ -2818,7 +2836,7 @@
     <t>Производительность по циклу на планировке объекта</t>
   </si>
   <si>
-    <t>thrцикл = 3600 / (Lпорож / v + Lгруз / (v × kгруз) + tопераций). Для single-leg-pallet-1: tопераций = 2 × tзахв. Для closed-pod-1: tопераций = 2H + 2 × (2H/3 + max(H/3; 2/v)), H = max(6; tзахв); Lпорож и Lгруз - суммарные пробеги двух физических перевозок на клиентскую заявку, включая подачу или возврат носителя.</t>
+    <t>thrцикл = 3600 / (Lпорож / v + Lгруз / (v × kгруз) + tопераций). Для single-leg-pallet-1: tопераций = 2 × tзахв. Для closed-pod-1: tопераций = (2 − dвнутр) / 2 × [2H + 2 × (2H/3 + max(H/3; 2/v))], H = max(6; tзахв), dвнутр — доля внутренних клиентских перевозок. Приёмка и отгрузка включают две физические перевозки с подачей или возвратом носителя; внутренняя перестановка — одну. Lпорож и Lгруз — средние суммарные пробеги на заявку с учётом состава потока.</t>
   </si>
   <si>
     <t>ед./ч; м; м/с; с</t>
@@ -2965,7 +2983,13 @@
     <t>Аналитическая производительность по циклу рассчитана для свободного маршрута. Для замкнутого цикла мобильного стеллажа closed-pod-1 выполнение нагрузки проверяется одной пространственной моделью: подача, подхват, перевозка, возврат, корпуса, встречное движение, защитные остановки и объезды. Для одиночной перевозки вилочным роботом или тягачом single-leg-pallet-1 используется аналитическая 2D-имитация очередей к точкам и зарядке; пространственную безопасность она не проверяет. Каждый результат относится к указанным входу и версии; люди и тормозной путь не моделируются.</t>
   </si>
   <si>
-    <t>Перевозка и порожний пробег рассчитаны по маршрутам указанной планировки. В closed-pod-1 это суммарные пробеги двух физических перевозок на одну клиентскую заявку, включая связанную подачу или возврат носителя. Без явного плана используется типовая геометрия из активной площади и ширины проходов; переданный план использует собственные стены, препятствия и граф. Демонстрационная планировка не является обследованным объектом.</t>
+    <t>Перевозка и порожний пробег рассчитаны по маршрутам указанной планировки и долям приёмки, отгрузки и внутренних перемещений. В closed-pod-1 приёмка и отгрузка включают две физические перевозки с подачей или возвратом носителя, внутренняя перестановка — одну перевозку между местами хранения. Служебные подачи и возвраты не добавляют клиентских паллет к выпуску. Без явного плана используется типовая геометрия; переданный план использует собственные стены, препятствия и граф. Демонстрационная планировка не является обследованным объектом.</t>
+  </si>
+  <si>
+    <t>Для внутренних перестановок начальная доля свободных мест задаётся нормативом simStorageVacancyShare (по умолчанию 10%, явная оценка, не обследование склада). Число свободных мест округляется вниз. Стеллаж резервирует свободное назначение и после перевозки освобождает исходное место; при нулевой свободной ёмкости перенос не подтверждается. Товарные остатки и наличие конкретной номенклатуры не моделируются.</t>
+  </si>
+  <si>
+    <t>Если за окно имитации не поступило клиентских заявок, нагрузка получает статус NOT_EVALUATED: нет наблюдений для подтверждения потока, минимального парка или пилота. Увеличьте окно или проверьте воспроизводимый нагруженный сценарий. Исторические входы без состава потока используют прежнее допущение 50/50 приёмки и отгрузки.</t>
   </si>
   <si>
     <t>Стоимость существующего парка погрузчиков и его обслуживания в исходных данных не задана, поэтому её экономия в эффект не входит — эффект занижен, оценка консервативна.</t>
@@ -4249,7 +4273,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K49"/>
+  <dimension ref="A1:K50"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -4266,16 +4290,16 @@
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>638</v>
+        <v>641</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>639</v>
+        <v>642</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>640</v>
+        <v>643</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>641</v>
+        <v>644</v>
       </c>
       <c r="E1" s="6" t="s">
         <v>100</v>
@@ -4284,16 +4308,16 @@
         <v>101</v>
       </c>
       <c r="G1" s="6" t="s">
-        <v>642</v>
+        <v>645</v>
       </c>
       <c r="H1" s="6" t="s">
-        <v>643</v>
+        <v>646</v>
       </c>
       <c r="I1" s="6" t="s">
         <v>482</v>
       </c>
       <c r="J1" s="6" t="s">
-        <v>644</v>
+        <v>647</v>
       </c>
       <c r="K1" s="6" t="s">
         <v>103</v>
@@ -4301,13 +4325,13 @@
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>645</v>
+        <v>648</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>646</v>
+        <v>649</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>647</v>
+        <v>650</v>
       </c>
       <c r="D2" s="4">
         <v>0.775</v>
@@ -4328,21 +4352,21 @@
         <v>487</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>648</v>
+        <v>651</v>
       </c>
       <c r="K2" s="3" t="s">
-        <v>649</v>
+        <v>652</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>645</v>
+        <v>648</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>650</v>
+        <v>653</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>651</v>
+        <v>654</v>
       </c>
       <c r="D3" s="4">
         <v>1</v>
@@ -4363,21 +4387,21 @@
         <v>269</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>652</v>
+        <v>655</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>653</v>
+        <v>656</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>645</v>
+        <v>648</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>654</v>
+        <v>657</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>655</v>
+        <v>658</v>
       </c>
       <c r="D4" s="4">
         <v>0.175</v>
@@ -4398,21 +4422,21 @@
         <v>487</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>656</v>
+        <v>659</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>657</v>
+        <v>660</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>645</v>
+        <v>648</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>658</v>
+        <v>661</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>659</v>
+        <v>662</v>
       </c>
       <c r="D5" s="4">
         <v>0.8</v>
@@ -4433,7 +4457,7 @@
         <v>261</v>
       </c>
       <c r="J5" s="3" t="s">
-        <v>660</v>
+        <v>663</v>
       </c>
       <c r="K5" s="4" t="s">
         <v>35</v>
@@ -4441,19 +4465,19 @@
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>645</v>
+        <v>648</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>661</v>
+        <v>664</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>662</v>
+        <v>665</v>
       </c>
       <c r="D6" s="4">
         <v>20</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>663</v>
+        <v>666</v>
       </c>
       <c r="F6" s="4">
         <v>20</v>
@@ -4468,7 +4492,7 @@
         <v>261</v>
       </c>
       <c r="J6" s="3" t="s">
-        <v>664</v>
+        <v>667</v>
       </c>
       <c r="K6" s="4" t="s">
         <v>35</v>
@@ -4476,19 +4500,19 @@
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>645</v>
+        <v>648</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>665</v>
+        <v>668</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>666</v>
+        <v>669</v>
       </c>
       <c r="D7" s="4">
         <v>45</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>663</v>
+        <v>666</v>
       </c>
       <c r="F7" s="4">
         <v>45</v>
@@ -4503,7 +4527,7 @@
         <v>261</v>
       </c>
       <c r="J7" s="3" t="s">
-        <v>667</v>
+        <v>670</v>
       </c>
       <c r="K7" s="4" t="s">
         <v>35</v>
@@ -4511,19 +4535,19 @@
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>645</v>
+        <v>648</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>668</v>
+        <v>671</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>669</v>
+        <v>672</v>
       </c>
       <c r="D8" s="4">
         <v>30</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>663</v>
+        <v>666</v>
       </c>
       <c r="F8" s="4">
         <v>30</v>
@@ -4538,7 +4562,7 @@
         <v>261</v>
       </c>
       <c r="J8" s="3" t="s">
-        <v>670</v>
+        <v>673</v>
       </c>
       <c r="K8" s="4" t="s">
         <v>35</v>
@@ -4546,13 +4570,13 @@
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>645</v>
+        <v>648</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>671</v>
+        <v>674</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>672</v>
+        <v>675</v>
       </c>
       <c r="D9" s="4">
         <v>1.5</v>
@@ -4573,7 +4597,7 @@
         <v>261</v>
       </c>
       <c r="J9" s="3" t="s">
-        <v>673</v>
+        <v>676</v>
       </c>
       <c r="K9" s="4" t="s">
         <v>35</v>
@@ -4581,13 +4605,13 @@
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>645</v>
+        <v>648</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>674</v>
+        <v>677</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>675</v>
+        <v>678</v>
       </c>
       <c r="D10" s="4">
         <v>5</v>
@@ -4608,7 +4632,7 @@
         <v>261</v>
       </c>
       <c r="J10" s="3" t="s">
-        <v>676</v>
+        <v>679</v>
       </c>
       <c r="K10" s="4" t="s">
         <v>35</v>
@@ -4616,13 +4640,13 @@
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>645</v>
+        <v>648</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>677</v>
+        <v>680</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>678</v>
+        <v>681</v>
       </c>
       <c r="D11" s="4">
         <v>3</v>
@@ -4643,7 +4667,7 @@
         <v>261</v>
       </c>
       <c r="J11" s="3" t="s">
-        <v>679</v>
+        <v>682</v>
       </c>
       <c r="K11" s="4" t="s">
         <v>35</v>
@@ -4651,13 +4675,13 @@
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
-        <v>680</v>
+        <v>683</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>681</v>
+        <v>684</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>682</v>
+        <v>685</v>
       </c>
       <c r="D12" s="4">
         <v>1.302</v>
@@ -4678,21 +4702,21 @@
         <v>487</v>
       </c>
       <c r="J12" s="3" t="s">
-        <v>683</v>
+        <v>686</v>
       </c>
       <c r="K12" s="4" t="s">
-        <v>684</v>
+        <v>687</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
-        <v>680</v>
+        <v>683</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>685</v>
+        <v>688</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>686</v>
+        <v>689</v>
       </c>
       <c r="D13" s="4">
         <v>0.5</v>
@@ -4713,7 +4737,7 @@
         <v>261</v>
       </c>
       <c r="J13" s="3" t="s">
-        <v>687</v>
+        <v>690</v>
       </c>
       <c r="K13" s="4" t="s">
         <v>35</v>
@@ -4721,13 +4745,13 @@
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
-        <v>680</v>
+        <v>683</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>688</v>
+        <v>691</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>689</v>
+        <v>692</v>
       </c>
       <c r="D14" s="4">
         <v>20</v>
@@ -4748,7 +4772,7 @@
         <v>261</v>
       </c>
       <c r="J14" s="3" t="s">
-        <v>690</v>
+        <v>693</v>
       </c>
       <c r="K14" s="4" t="s">
         <v>35</v>
@@ -4756,13 +4780,13 @@
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
-        <v>680</v>
+        <v>683</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>691</v>
+        <v>694</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>692</v>
+        <v>695</v>
       </c>
       <c r="D15" s="4">
         <v>1973</v>
@@ -4783,7 +4807,7 @@
         <v>261</v>
       </c>
       <c r="J15" s="3" t="s">
-        <v>693</v>
+        <v>696</v>
       </c>
       <c r="K15" s="4" t="s">
         <v>35</v>
@@ -4794,10 +4818,10 @@
         <v>31</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>694</v>
+        <v>697</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>695</v>
+        <v>698</v>
       </c>
       <c r="D16" s="4">
         <v>0.1</v>
@@ -4818,10 +4842,10 @@
         <v>487</v>
       </c>
       <c r="J16" s="3" t="s">
-        <v>696</v>
+        <v>699</v>
       </c>
       <c r="K16" s="3" t="s">
-        <v>697</v>
+        <v>700</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
@@ -4829,10 +4853,10 @@
         <v>31</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>698</v>
+        <v>701</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>699</v>
+        <v>702</v>
       </c>
       <c r="D17" s="4">
         <v>1000000</v>
@@ -4853,10 +4877,10 @@
         <v>491</v>
       </c>
       <c r="J17" s="3" t="s">
-        <v>700</v>
+        <v>703</v>
       </c>
       <c r="K17" s="3" t="s">
-        <v>701</v>
+        <v>704</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
@@ -4864,10 +4888,10 @@
         <v>31</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>702</v>
+        <v>705</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>703</v>
+        <v>706</v>
       </c>
       <c r="D18" s="4">
         <v>1250000</v>
@@ -4888,10 +4912,10 @@
         <v>491</v>
       </c>
       <c r="J18" s="3" t="s">
-        <v>704</v>
+        <v>707</v>
       </c>
       <c r="K18" s="3" t="s">
-        <v>705</v>
+        <v>708</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
@@ -4899,10 +4923,10 @@
         <v>31</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>706</v>
+        <v>709</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>707</v>
+        <v>710</v>
       </c>
       <c r="D19" s="4">
         <v>100000</v>
@@ -4923,10 +4947,10 @@
         <v>491</v>
       </c>
       <c r="J19" s="3" t="s">
-        <v>708</v>
+        <v>711</v>
       </c>
       <c r="K19" s="3" t="s">
-        <v>709</v>
+        <v>712</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.25">
@@ -4934,10 +4958,10 @@
         <v>31</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>710</v>
+        <v>713</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>711</v>
+        <v>714</v>
       </c>
       <c r="D20" s="4">
         <v>150000</v>
@@ -4958,7 +4982,7 @@
         <v>261</v>
       </c>
       <c r="J20" s="3" t="s">
-        <v>712</v>
+        <v>715</v>
       </c>
       <c r="K20" s="4" t="s">
         <v>35</v>
@@ -4969,10 +4993,10 @@
         <v>31</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>713</v>
+        <v>716</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>714</v>
+        <v>717</v>
       </c>
       <c r="D21" s="4">
         <v>300000</v>
@@ -4993,10 +5017,10 @@
         <v>491</v>
       </c>
       <c r="J21" s="3" t="s">
-        <v>715</v>
+        <v>718</v>
       </c>
       <c r="K21" s="3" t="s">
-        <v>716</v>
+        <v>719</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.25">
@@ -5004,16 +5028,16 @@
         <v>31</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>717</v>
+        <v>720</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>718</v>
+        <v>721</v>
       </c>
       <c r="D22" s="4">
         <v>150</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>719</v>
+        <v>722</v>
       </c>
       <c r="F22" s="4">
         <v>150</v>
@@ -5028,7 +5052,7 @@
         <v>261</v>
       </c>
       <c r="J22" s="3" t="s">
-        <v>720</v>
+        <v>723</v>
       </c>
       <c r="K22" s="4" t="s">
         <v>35</v>
@@ -5036,13 +5060,13 @@
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" s="4" t="s">
-        <v>721</v>
+        <v>724</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>723</v>
+        <v>726</v>
       </c>
       <c r="D23" s="4">
         <v>0.12</v>
@@ -5063,21 +5087,21 @@
         <v>491</v>
       </c>
       <c r="J23" s="3" t="s">
-        <v>724</v>
+        <v>727</v>
       </c>
       <c r="K23" s="3" t="s">
-        <v>725</v>
+        <v>728</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" s="4" t="s">
-        <v>721</v>
+        <v>724</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>726</v>
+        <v>729</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>727</v>
+        <v>730</v>
       </c>
       <c r="D24" s="4">
         <v>0.02</v>
@@ -5098,7 +5122,7 @@
         <v>261</v>
       </c>
       <c r="J24" s="3" t="s">
-        <v>728</v>
+        <v>731</v>
       </c>
       <c r="K24" s="4" t="s">
         <v>35</v>
@@ -5106,13 +5130,13 @@
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" s="4" t="s">
-        <v>721</v>
+        <v>724</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>729</v>
+        <v>732</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>730</v>
+        <v>733</v>
       </c>
       <c r="D25" s="4">
         <v>0.01</v>
@@ -5133,7 +5157,7 @@
         <v>261</v>
       </c>
       <c r="J25" s="3" t="s">
-        <v>731</v>
+        <v>734</v>
       </c>
       <c r="K25" s="4" t="s">
         <v>35</v>
@@ -5141,13 +5165,13 @@
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" s="4" t="s">
-        <v>721</v>
+        <v>724</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>732</v>
+        <v>735</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>733</v>
+        <v>736</v>
       </c>
       <c r="D26" s="4">
         <v>4</v>
@@ -5168,21 +5192,21 @@
         <v>487</v>
       </c>
       <c r="J26" s="3" t="s">
-        <v>734</v>
+        <v>737</v>
       </c>
       <c r="K26" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" s="4" t="s">
-        <v>721</v>
+        <v>724</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>736</v>
+        <v>739</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>737</v>
+        <v>740</v>
       </c>
       <c r="D27" s="4">
         <v>0.1</v>
@@ -5203,7 +5227,7 @@
         <v>261</v>
       </c>
       <c r="J27" s="3" t="s">
-        <v>738</v>
+        <v>741</v>
       </c>
       <c r="K27" s="4" t="s">
         <v>35</v>
@@ -5211,13 +5235,13 @@
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" s="4" t="s">
-        <v>721</v>
+        <v>724</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>739</v>
+        <v>742</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>740</v>
+        <v>743</v>
       </c>
       <c r="D28" s="4">
         <v>0.4</v>
@@ -5238,7 +5262,7 @@
         <v>261</v>
       </c>
       <c r="J28" s="3" t="s">
-        <v>741</v>
+        <v>744</v>
       </c>
       <c r="K28" s="4" t="s">
         <v>35</v>
@@ -5246,19 +5270,19 @@
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" s="4" t="s">
-        <v>721</v>
+        <v>724</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>742</v>
+        <v>745</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>743</v>
+        <v>746</v>
       </c>
       <c r="D29" s="4">
         <v>9</v>
       </c>
       <c r="E29" s="4" t="s">
-        <v>744</v>
+        <v>747</v>
       </c>
       <c r="F29" s="4">
         <v>9</v>
@@ -5273,7 +5297,7 @@
         <v>261</v>
       </c>
       <c r="J29" s="3" t="s">
-        <v>745</v>
+        <v>748</v>
       </c>
       <c r="K29" s="4" t="s">
         <v>35</v>
@@ -5281,13 +5305,13 @@
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" s="4" t="s">
-        <v>721</v>
+        <v>724</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>746</v>
+        <v>749</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>747</v>
+        <v>750</v>
       </c>
       <c r="D30" s="4">
         <v>12000</v>
@@ -5308,7 +5332,7 @@
         <v>261</v>
       </c>
       <c r="J30" s="3" t="s">
-        <v>748</v>
+        <v>751</v>
       </c>
       <c r="K30" s="4" t="s">
         <v>35</v>
@@ -5316,19 +5340,19 @@
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" s="4" t="s">
-        <v>721</v>
+        <v>724</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>749</v>
+        <v>752</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>750</v>
+        <v>753</v>
       </c>
       <c r="D31" s="4">
         <v>0.052</v>
       </c>
       <c r="E31" s="4" t="s">
-        <v>751</v>
+        <v>754</v>
       </c>
       <c r="F31" s="4">
         <v>0.052</v>
@@ -5343,21 +5367,21 @@
         <v>269</v>
       </c>
       <c r="J31" s="3" t="s">
-        <v>752</v>
+        <v>755</v>
       </c>
       <c r="K31" s="3" t="s">
-        <v>753</v>
+        <v>756</v>
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" s="4" t="s">
-        <v>754</v>
+        <v>757</v>
       </c>
       <c r="B32" s="4" t="s">
         <v>555</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>755</v>
+        <v>758</v>
       </c>
       <c r="D32" s="4">
         <v>0.12</v>
@@ -5375,10 +5399,10 @@
         <v>0.2</v>
       </c>
       <c r="I32" s="4" t="s">
-        <v>756</v>
+        <v>759</v>
       </c>
       <c r="J32" s="3" t="s">
-        <v>757</v>
+        <v>760</v>
       </c>
       <c r="K32" s="4" t="s">
         <v>35</v>
@@ -5386,13 +5410,13 @@
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" s="4" t="s">
-        <v>754</v>
+        <v>757</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>758</v>
+        <v>761</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>759</v>
+        <v>762</v>
       </c>
       <c r="D33" s="4">
         <v>7</v>
@@ -5413,7 +5437,7 @@
         <v>261</v>
       </c>
       <c r="J33" s="3" t="s">
-        <v>760</v>
+        <v>763</v>
       </c>
       <c r="K33" s="4" t="s">
         <v>35</v>
@@ -5421,13 +5445,13 @@
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" s="4" t="s">
-        <v>754</v>
+        <v>757</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>761</v>
+        <v>764</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>762</v>
+        <v>765</v>
       </c>
       <c r="D34" s="4">
         <v>5</v>
@@ -5445,13 +5469,13 @@
         <v>30</v>
       </c>
       <c r="I34" s="4" t="s">
-        <v>763</v>
+        <v>766</v>
       </c>
       <c r="J34" s="3" t="s">
-        <v>764</v>
+        <v>767</v>
       </c>
       <c r="K34" s="4" t="s">
-        <v>765</v>
+        <v>768</v>
       </c>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.25">
@@ -5459,10 +5483,10 @@
         <v>37</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>766</v>
+        <v>769</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>767</v>
+        <v>770</v>
       </c>
       <c r="D35" s="4">
         <v>3</v>
@@ -5480,13 +5504,13 @@
         <v>35</v>
       </c>
       <c r="I35" s="4" t="s">
-        <v>763</v>
+        <v>766</v>
       </c>
       <c r="J35" s="3" t="s">
-        <v>768</v>
+        <v>771</v>
       </c>
       <c r="K35" s="4" t="s">
-        <v>769</v>
+        <v>772</v>
       </c>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.25">
@@ -5494,10 +5518,10 @@
         <v>37</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>770</v>
+        <v>773</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>771</v>
+        <v>774</v>
       </c>
       <c r="D36" s="4">
         <v>5</v>
@@ -5515,13 +5539,13 @@
         <v>35</v>
       </c>
       <c r="I36" s="4" t="s">
-        <v>763</v>
+        <v>766</v>
       </c>
       <c r="J36" s="3" t="s">
+        <v>775</v>
+      </c>
+      <c r="K36" s="4" t="s">
         <v>772</v>
-      </c>
-      <c r="K36" s="4" t="s">
-        <v>769</v>
       </c>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.25">
@@ -5529,10 +5553,10 @@
         <v>37</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>773</v>
+        <v>776</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>774</v>
+        <v>777</v>
       </c>
       <c r="D37" s="4">
         <v>0.2</v>
@@ -5550,10 +5574,10 @@
         <v>1</v>
       </c>
       <c r="I37" s="4" t="s">
-        <v>756</v>
+        <v>759</v>
       </c>
       <c r="J37" s="3" t="s">
-        <v>775</v>
+        <v>778</v>
       </c>
       <c r="K37" s="4" t="s">
         <v>35</v>
@@ -5564,10 +5588,10 @@
         <v>47</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>776</v>
+        <v>779</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>777</v>
+        <v>780</v>
       </c>
       <c r="D38" s="4">
         <v>0.97</v>
@@ -5588,7 +5612,7 @@
         <v>261</v>
       </c>
       <c r="J38" s="3" t="s">
-        <v>778</v>
+        <v>781</v>
       </c>
       <c r="K38" s="4" t="s">
         <v>35</v>
@@ -5599,16 +5623,16 @@
         <v>47</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>779</v>
+        <v>782</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>780</v>
+        <v>783</v>
       </c>
       <c r="D39" s="4">
         <v>10</v>
       </c>
       <c r="E39" s="4" t="s">
-        <v>781</v>
+        <v>784</v>
       </c>
       <c r="F39" s="4">
         <v>10</v>
@@ -5623,7 +5647,7 @@
         <v>261</v>
       </c>
       <c r="J39" s="3" t="s">
-        <v>782</v>
+        <v>785</v>
       </c>
       <c r="K39" s="4" t="s">
         <v>35</v>
@@ -5634,10 +5658,10 @@
         <v>47</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>783</v>
+        <v>786</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>784</v>
+        <v>787</v>
       </c>
       <c r="D40" s="4">
         <v>0.4</v>
@@ -5658,7 +5682,7 @@
         <v>261</v>
       </c>
       <c r="J40" s="3" t="s">
-        <v>785</v>
+        <v>788</v>
       </c>
       <c r="K40" s="4" t="s">
         <v>35</v>
@@ -5668,32 +5692,32 @@
       <c r="A41" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="B41" s="4" t="s">
-        <v>786</v>
+      <c r="B41" s="3" t="s">
+        <v>789</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>787</v>
+        <v>790</v>
       </c>
       <c r="D41" s="4">
-        <v>15</v>
+        <v>0.1</v>
       </c>
       <c r="E41" s="4" t="s">
-        <v>781</v>
+        <v>600</v>
       </c>
       <c r="F41" s="4">
-        <v>15</v>
+        <v>0.1</v>
       </c>
       <c r="G41" s="4">
         <v>0</v>
       </c>
       <c r="H41" s="4">
-        <v>60</v>
+        <v>0.9</v>
       </c>
       <c r="I41" s="4" t="s">
         <v>261</v>
       </c>
       <c r="J41" s="3" t="s">
-        <v>788</v>
+        <v>791</v>
       </c>
       <c r="K41" s="4" t="s">
         <v>35</v>
@@ -5704,31 +5728,31 @@
         <v>47</v>
       </c>
       <c r="B42" s="4" t="s">
-        <v>789</v>
+        <v>792</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>790</v>
+        <v>793</v>
       </c>
       <c r="D42" s="4">
-        <v>120</v>
+        <v>15</v>
       </c>
       <c r="E42" s="4" t="s">
-        <v>781</v>
+        <v>784</v>
       </c>
       <c r="F42" s="4">
-        <v>120</v>
+        <v>15</v>
       </c>
       <c r="G42" s="4">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="H42" s="4">
-        <v>480</v>
+        <v>60</v>
       </c>
       <c r="I42" s="4" t="s">
         <v>261</v>
       </c>
       <c r="J42" s="3" t="s">
-        <v>791</v>
+        <v>794</v>
       </c>
       <c r="K42" s="4" t="s">
         <v>35</v>
@@ -5738,32 +5762,32 @@
       <c r="A43" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="B43" s="3" t="s">
-        <v>792</v>
+      <c r="B43" s="4" t="s">
+        <v>795</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>793</v>
+        <v>796</v>
       </c>
       <c r="D43" s="4">
-        <v>0.2</v>
+        <v>120</v>
       </c>
       <c r="E43" s="4" t="s">
-        <v>600</v>
+        <v>784</v>
       </c>
       <c r="F43" s="4">
-        <v>0.2</v>
+        <v>120</v>
       </c>
       <c r="G43" s="4">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="H43" s="4">
-        <v>0.95</v>
+        <v>480</v>
       </c>
       <c r="I43" s="4" t="s">
         <v>261</v>
       </c>
       <c r="J43" s="3" t="s">
-        <v>794</v>
+        <v>797</v>
       </c>
       <c r="K43" s="4" t="s">
         <v>35</v>
@@ -5774,31 +5798,31 @@
         <v>47</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>795</v>
+        <v>798</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>796</v>
+        <v>799</v>
       </c>
       <c r="D44" s="4">
-        <v>0.9</v>
+        <v>0.2</v>
       </c>
       <c r="E44" s="4" t="s">
         <v>600</v>
       </c>
       <c r="F44" s="4">
-        <v>0.9</v>
+        <v>0.2</v>
       </c>
       <c r="G44" s="4">
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="H44" s="4">
-        <v>1</v>
+        <v>0.95</v>
       </c>
       <c r="I44" s="4" t="s">
         <v>261</v>
       </c>
       <c r="J44" s="3" t="s">
-        <v>797</v>
+        <v>800</v>
       </c>
       <c r="K44" s="4" t="s">
         <v>35</v>
@@ -5806,34 +5830,34 @@
     </row>
     <row r="45" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A45" s="4" t="s">
-        <v>798</v>
-      </c>
-      <c r="B45" s="4" t="s">
-        <v>799</v>
+        <v>47</v>
+      </c>
+      <c r="B45" s="3" t="s">
+        <v>801</v>
       </c>
       <c r="C45" s="4" t="s">
-        <v>800</v>
+        <v>802</v>
       </c>
       <c r="D45" s="4">
-        <v>0.4</v>
+        <v>0.9</v>
       </c>
       <c r="E45" s="4" t="s">
         <v>600</v>
       </c>
       <c r="F45" s="4">
-        <v>0.4</v>
+        <v>0.9</v>
       </c>
       <c r="G45" s="4">
-        <v>0</v>
+        <v>0.05</v>
       </c>
       <c r="H45" s="4">
         <v>1</v>
       </c>
       <c r="I45" s="4" t="s">
-        <v>756</v>
+        <v>261</v>
       </c>
       <c r="J45" s="3" t="s">
-        <v>801</v>
+        <v>803</v>
       </c>
       <c r="K45" s="4" t="s">
         <v>35</v>
@@ -5841,22 +5865,22 @@
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A46" s="4" t="s">
-        <v>798</v>
+        <v>804</v>
       </c>
       <c r="B46" s="4" t="s">
-        <v>802</v>
+        <v>805</v>
       </c>
       <c r="C46" s="4" t="s">
-        <v>803</v>
+        <v>806</v>
       </c>
       <c r="D46" s="4">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="E46" s="4" t="s">
         <v>600</v>
       </c>
       <c r="F46" s="4">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="G46" s="4">
         <v>0</v>
@@ -5865,10 +5889,10 @@
         <v>1</v>
       </c>
       <c r="I46" s="4" t="s">
-        <v>756</v>
+        <v>759</v>
       </c>
       <c r="J46" s="3" t="s">
-        <v>804</v>
+        <v>807</v>
       </c>
       <c r="K46" s="4" t="s">
         <v>35</v>
@@ -5876,22 +5900,22 @@
     </row>
     <row r="47" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A47" s="4" t="s">
-        <v>798</v>
+        <v>804</v>
       </c>
       <c r="B47" s="4" t="s">
-        <v>805</v>
+        <v>808</v>
       </c>
       <c r="C47" s="4" t="s">
-        <v>806</v>
+        <v>809</v>
       </c>
       <c r="D47" s="4">
-        <v>0.15</v>
+        <v>0.2</v>
       </c>
       <c r="E47" s="4" t="s">
         <v>600</v>
       </c>
       <c r="F47" s="4">
-        <v>0.15</v>
+        <v>0.2</v>
       </c>
       <c r="G47" s="4">
         <v>0</v>
@@ -5900,10 +5924,10 @@
         <v>1</v>
       </c>
       <c r="I47" s="4" t="s">
-        <v>756</v>
+        <v>759</v>
       </c>
       <c r="J47" s="3" t="s">
-        <v>807</v>
+        <v>810</v>
       </c>
       <c r="K47" s="4" t="s">
         <v>35</v>
@@ -5911,13 +5935,13 @@
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A48" s="4" t="s">
-        <v>798</v>
+        <v>804</v>
       </c>
       <c r="B48" s="4" t="s">
-        <v>808</v>
+        <v>811</v>
       </c>
       <c r="C48" s="4" t="s">
-        <v>809</v>
+        <v>812</v>
       </c>
       <c r="D48" s="4">
         <v>0.15</v>
@@ -5935,10 +5959,10 @@
         <v>1</v>
       </c>
       <c r="I48" s="4" t="s">
-        <v>756</v>
+        <v>759</v>
       </c>
       <c r="J48" s="3" t="s">
-        <v>810</v>
+        <v>813</v>
       </c>
       <c r="K48" s="4" t="s">
         <v>35</v>
@@ -5946,22 +5970,22 @@
     </row>
     <row r="49" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A49" s="4" t="s">
-        <v>798</v>
+        <v>804</v>
       </c>
       <c r="B49" s="4" t="s">
-        <v>811</v>
+        <v>814</v>
       </c>
       <c r="C49" s="4" t="s">
-        <v>812</v>
+        <v>815</v>
       </c>
       <c r="D49" s="4">
-        <v>0.1</v>
+        <v>0.15</v>
       </c>
       <c r="E49" s="4" t="s">
         <v>600</v>
       </c>
       <c r="F49" s="4">
-        <v>0.1</v>
+        <v>0.15</v>
       </c>
       <c r="G49" s="4">
         <v>0</v>
@@ -5970,12 +5994,47 @@
         <v>1</v>
       </c>
       <c r="I49" s="4" t="s">
-        <v>756</v>
+        <v>759</v>
       </c>
       <c r="J49" s="3" t="s">
-        <v>813</v>
+        <v>816</v>
       </c>
       <c r="K49" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A50" s="4" t="s">
+        <v>804</v>
+      </c>
+      <c r="B50" s="4" t="s">
+        <v>817</v>
+      </c>
+      <c r="C50" s="4" t="s">
+        <v>818</v>
+      </c>
+      <c r="D50" s="4">
+        <v>0.1</v>
+      </c>
+      <c r="E50" s="4" t="s">
+        <v>600</v>
+      </c>
+      <c r="F50" s="4">
+        <v>0.1</v>
+      </c>
+      <c r="G50" s="4">
+        <v>0</v>
+      </c>
+      <c r="H50" s="4">
+        <v>1</v>
+      </c>
+      <c r="I50" s="4" t="s">
+        <v>759</v>
+      </c>
+      <c r="J50" s="3" t="s">
+        <v>819</v>
+      </c>
+      <c r="K50" s="4" t="s">
         <v>35</v>
       </c>
     </row>
@@ -6004,7 +6063,7 @@
         <v>285</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>814</v>
+        <v>820</v>
       </c>
       <c r="C1" s="6" t="s">
         <v>99</v>
@@ -6013,16 +6072,16 @@
         <v>482</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>815</v>
+        <v>821</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>816</v>
+        <v>822</v>
       </c>
       <c r="G1" s="6" t="s">
-        <v>817</v>
+        <v>823</v>
       </c>
       <c r="H1" s="6" t="s">
-        <v>818</v>
+        <v>824</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
@@ -6030,10 +6089,10 @@
         <v>307</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>819</v>
+        <v>825</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>820</v>
+        <v>826</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>487</v>
@@ -6042,13 +6101,13 @@
         <v>50</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>821</v>
+        <v>827</v>
       </c>
       <c r="G2" s="4" t="s">
         <v>35</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>822</v>
+        <v>828</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -6056,7 +6115,7 @@
         <v>307</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>823</v>
+        <v>829</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>307</v>
@@ -6068,13 +6127,13 @@
         <v>50</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>821</v>
+        <v>827</v>
       </c>
       <c r="G3" s="4" t="s">
         <v>35</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>822</v>
+        <v>828</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -6082,19 +6141,19 @@
         <v>307</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>824</v>
+        <v>830</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>825</v>
+        <v>831</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>756</v>
+        <v>759</v>
       </c>
       <c r="E4" s="4" t="s">
         <v>50</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>826</v>
+        <v>832</v>
       </c>
       <c r="G4" s="4" t="s">
         <v>35</v>
@@ -6108,10 +6167,10 @@
         <v>307</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>827</v>
+        <v>833</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>828</v>
+        <v>834</v>
       </c>
       <c r="D5" s="4" t="s">
         <v>487</v>
@@ -6120,13 +6179,13 @@
         <v>50</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>821</v>
+        <v>827</v>
       </c>
       <c r="G5" s="4" t="s">
         <v>35</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>822</v>
+        <v>828</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
@@ -6134,10 +6193,10 @@
         <v>307</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>829</v>
+        <v>835</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>830</v>
+        <v>836</v>
       </c>
       <c r="D6" s="4" t="s">
         <v>491</v>
@@ -6146,10 +6205,10 @@
         <v>296</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>826</v>
+        <v>832</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>831</v>
+        <v>837</v>
       </c>
       <c r="H6" s="4" t="s">
         <v>35</v>
@@ -6160,10 +6219,10 @@
         <v>307</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>832</v>
+        <v>838</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>833</v>
+        <v>839</v>
       </c>
       <c r="D7" s="4" t="s">
         <v>487</v>
@@ -6172,13 +6231,13 @@
         <v>50</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>821</v>
+        <v>827</v>
       </c>
       <c r="G7" s="4" t="s">
         <v>35</v>
       </c>
       <c r="H7" s="4" t="s">
-        <v>822</v>
+        <v>828</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -6186,10 +6245,10 @@
         <v>307</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>834</v>
+        <v>840</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>835</v>
+        <v>841</v>
       </c>
       <c r="D8" s="4" t="s">
         <v>487</v>
@@ -6198,13 +6257,13 @@
         <v>50</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>821</v>
+        <v>827</v>
       </c>
       <c r="G8" s="4" t="s">
         <v>35</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>836</v>
+        <v>842</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
@@ -6212,10 +6271,10 @@
         <v>307</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>837</v>
+        <v>843</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>838</v>
+        <v>844</v>
       </c>
       <c r="D9" s="4" t="s">
         <v>487</v>
@@ -6224,13 +6283,13 @@
         <v>50</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>821</v>
+        <v>827</v>
       </c>
       <c r="G9" s="4" t="s">
         <v>35</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>836</v>
+        <v>842</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
@@ -6238,10 +6297,10 @@
         <v>307</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>839</v>
+        <v>845</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>840</v>
+        <v>846</v>
       </c>
       <c r="D10" s="4" t="s">
         <v>487</v>
@@ -6250,13 +6309,13 @@
         <v>296</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>821</v>
+        <v>827</v>
       </c>
       <c r="G10" s="4" t="s">
         <v>35</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>836</v>
+        <v>842</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
@@ -6264,10 +6323,10 @@
         <v>307</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>841</v>
+        <v>847</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>842</v>
+        <v>848</v>
       </c>
       <c r="D11" s="4" t="s">
         <v>487</v>
@@ -6276,13 +6335,13 @@
         <v>50</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>821</v>
+        <v>827</v>
       </c>
       <c r="G11" s="4" t="s">
         <v>35</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>836</v>
+        <v>842</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
@@ -6290,10 +6349,10 @@
         <v>307</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>843</v>
+        <v>849</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>844</v>
+        <v>850</v>
       </c>
       <c r="D12" s="4" t="s">
         <v>487</v>
@@ -6302,13 +6361,13 @@
         <v>50</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>821</v>
+        <v>827</v>
       </c>
       <c r="G12" s="4" t="s">
         <v>35</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>836</v>
+        <v>842</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
@@ -6316,10 +6375,10 @@
         <v>307</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>845</v>
+        <v>851</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>846</v>
+        <v>852</v>
       </c>
       <c r="D13" s="4" t="s">
         <v>487</v>
@@ -6328,13 +6387,13 @@
         <v>50</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>821</v>
+        <v>827</v>
       </c>
       <c r="G13" s="4" t="s">
         <v>35</v>
       </c>
       <c r="H13" s="3" t="s">
-        <v>836</v>
+        <v>842</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
@@ -6342,10 +6401,10 @@
         <v>307</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>847</v>
+        <v>853</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>848</v>
+        <v>854</v>
       </c>
       <c r="D14" s="4" t="s">
         <v>487</v>
@@ -6354,13 +6413,13 @@
         <v>50</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>821</v>
+        <v>827</v>
       </c>
       <c r="G14" s="4" t="s">
         <v>35</v>
       </c>
       <c r="H14" s="3" t="s">
-        <v>836</v>
+        <v>842</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
@@ -6368,10 +6427,10 @@
         <v>307</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>849</v>
+        <v>855</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>850</v>
+        <v>856</v>
       </c>
       <c r="D15" s="4" t="s">
         <v>487</v>
@@ -6380,13 +6439,13 @@
         <v>50</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>821</v>
+        <v>827</v>
       </c>
       <c r="G15" s="4" t="s">
         <v>35</v>
       </c>
       <c r="H15" s="3" t="s">
-        <v>836</v>
+        <v>842</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
@@ -6394,10 +6453,10 @@
         <v>307</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>851</v>
+        <v>857</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>852</v>
+        <v>858</v>
       </c>
       <c r="D16" s="4" t="s">
         <v>487</v>
@@ -6406,13 +6465,13 @@
         <v>50</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>821</v>
+        <v>827</v>
       </c>
       <c r="G16" s="4" t="s">
         <v>35</v>
       </c>
       <c r="H16" s="3" t="s">
-        <v>836</v>
+        <v>842</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
@@ -6420,10 +6479,10 @@
         <v>307</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>853</v>
+        <v>859</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>854</v>
+        <v>860</v>
       </c>
       <c r="D17" s="4" t="s">
         <v>487</v>
@@ -6432,13 +6491,13 @@
         <v>50</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>821</v>
+        <v>827</v>
       </c>
       <c r="G17" s="4" t="s">
         <v>35</v>
       </c>
       <c r="H17" s="3" t="s">
-        <v>836</v>
+        <v>842</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
@@ -6446,10 +6505,10 @@
         <v>307</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>855</v>
+        <v>861</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>856</v>
+        <v>862</v>
       </c>
       <c r="D18" s="4" t="s">
         <v>487</v>
@@ -6458,13 +6517,13 @@
         <v>50</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>821</v>
+        <v>827</v>
       </c>
       <c r="G18" s="4" t="s">
         <v>35</v>
       </c>
       <c r="H18" s="3" t="s">
-        <v>836</v>
+        <v>842</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
@@ -6472,10 +6531,10 @@
         <v>307</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>857</v>
+        <v>863</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>858</v>
+        <v>864</v>
       </c>
       <c r="D19" s="4" t="s">
         <v>491</v>
@@ -6484,10 +6543,10 @@
         <v>296</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>826</v>
+        <v>832</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>859</v>
+        <v>865</v>
       </c>
       <c r="H19" s="4" t="s">
         <v>35</v>
@@ -6498,10 +6557,10 @@
         <v>307</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>860</v>
+        <v>866</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>861</v>
+        <v>867</v>
       </c>
       <c r="D20" s="4" t="s">
         <v>491</v>
@@ -6510,10 +6569,10 @@
         <v>296</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>826</v>
+        <v>832</v>
       </c>
       <c r="G20" s="4" t="s">
-        <v>831</v>
+        <v>837</v>
       </c>
       <c r="H20" s="4" t="s">
         <v>35</v>
@@ -6524,10 +6583,10 @@
         <v>307</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>862</v>
+        <v>868</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>863</v>
+        <v>869</v>
       </c>
       <c r="D21" s="4" t="s">
         <v>487</v>
@@ -6536,13 +6595,13 @@
         <v>50</v>
       </c>
       <c r="F21" s="4" t="s">
-        <v>821</v>
+        <v>827</v>
       </c>
       <c r="G21" s="4" t="s">
         <v>35</v>
       </c>
       <c r="H21" s="3" t="s">
-        <v>836</v>
+        <v>842</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
@@ -6550,10 +6609,10 @@
         <v>307</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>864</v>
+        <v>870</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>865</v>
+        <v>871</v>
       </c>
       <c r="D22" s="4" t="s">
         <v>491</v>
@@ -6562,10 +6621,10 @@
         <v>296</v>
       </c>
       <c r="F22" s="4" t="s">
-        <v>826</v>
+        <v>832</v>
       </c>
       <c r="G22" s="4" t="s">
-        <v>831</v>
+        <v>837</v>
       </c>
       <c r="H22" s="4" t="s">
         <v>35</v>
@@ -6576,10 +6635,10 @@
         <v>307</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>866</v>
+        <v>872</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>865</v>
+        <v>871</v>
       </c>
       <c r="D23" s="4" t="s">
         <v>491</v>
@@ -6588,10 +6647,10 @@
         <v>296</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>826</v>
+        <v>832</v>
       </c>
       <c r="G23" s="4" t="s">
-        <v>831</v>
+        <v>837</v>
       </c>
       <c r="H23" s="4" t="s">
         <v>35</v>
@@ -6602,10 +6661,10 @@
         <v>307</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>867</v>
+        <v>873</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>868</v>
+        <v>874</v>
       </c>
       <c r="D24" s="4" t="s">
         <v>487</v>
@@ -6614,13 +6673,13 @@
         <v>296</v>
       </c>
       <c r="F24" s="4" t="s">
-        <v>821</v>
+        <v>827</v>
       </c>
       <c r="G24" s="4" t="s">
         <v>35</v>
       </c>
       <c r="H24" s="4" t="s">
-        <v>822</v>
+        <v>828</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
@@ -6628,10 +6687,10 @@
         <v>307</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>869</v>
+        <v>875</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>870</v>
+        <v>876</v>
       </c>
       <c r="D25" s="4" t="s">
         <v>491</v>
@@ -6640,10 +6699,10 @@
         <v>50</v>
       </c>
       <c r="F25" s="4" t="s">
-        <v>826</v>
+        <v>832</v>
       </c>
       <c r="G25" s="4" t="s">
-        <v>871</v>
+        <v>877</v>
       </c>
       <c r="H25" s="4" t="s">
         <v>35</v>
@@ -6654,10 +6713,10 @@
         <v>307</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>872</v>
+        <v>878</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>873</v>
+        <v>879</v>
       </c>
       <c r="D26" s="4" t="s">
         <v>491</v>
@@ -6666,10 +6725,10 @@
         <v>50</v>
       </c>
       <c r="F26" s="4" t="s">
-        <v>826</v>
+        <v>832</v>
       </c>
       <c r="G26" s="4" t="s">
-        <v>874</v>
+        <v>880</v>
       </c>
       <c r="H26" s="4" t="s">
         <v>35</v>
@@ -6683,7 +6742,7 @@
         <v>519</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>875</v>
+        <v>881</v>
       </c>
       <c r="D27" s="4" t="s">
         <v>491</v>
@@ -6692,10 +6751,10 @@
         <v>296</v>
       </c>
       <c r="F27" s="4" t="s">
-        <v>826</v>
+        <v>832</v>
       </c>
       <c r="G27" s="4" t="s">
-        <v>874</v>
+        <v>880</v>
       </c>
       <c r="H27" s="4" t="s">
         <v>35</v>
@@ -6706,10 +6765,10 @@
         <v>307</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>876</v>
+        <v>882</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>877</v>
+        <v>883</v>
       </c>
       <c r="D28" s="4" t="s">
         <v>491</v>
@@ -6718,10 +6777,10 @@
         <v>296</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>826</v>
+        <v>832</v>
       </c>
       <c r="G28" s="4" t="s">
-        <v>831</v>
+        <v>837</v>
       </c>
       <c r="H28" s="4" t="s">
         <v>35</v>
@@ -6735,7 +6794,7 @@
         <v>615</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>878</v>
+        <v>884</v>
       </c>
       <c r="D29" s="4" t="s">
         <v>491</v>
@@ -6744,10 +6803,10 @@
         <v>50</v>
       </c>
       <c r="F29" s="4" t="s">
-        <v>826</v>
+        <v>832</v>
       </c>
       <c r="G29" s="4" t="s">
-        <v>879</v>
+        <v>885</v>
       </c>
       <c r="H29" s="4" t="s">
         <v>35</v>
@@ -6758,10 +6817,10 @@
         <v>307</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>732</v>
+        <v>735</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>880</v>
+        <v>886</v>
       </c>
       <c r="D30" s="4" t="s">
         <v>491</v>
@@ -6770,10 +6829,10 @@
         <v>50</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>826</v>
+        <v>832</v>
       </c>
       <c r="G30" s="4" t="s">
-        <v>881</v>
+        <v>887</v>
       </c>
       <c r="H30" s="4" t="s">
         <v>35</v>
@@ -6784,19 +6843,19 @@
         <v>307</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>882</v>
+        <v>888</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>883</v>
+        <v>889</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>756</v>
+        <v>759</v>
       </c>
       <c r="E31" s="4" t="s">
         <v>50</v>
       </c>
       <c r="F31" s="4" t="s">
-        <v>826</v>
+        <v>832</v>
       </c>
       <c r="G31" s="4" t="s">
         <v>35</v>
@@ -6810,10 +6869,10 @@
         <v>307</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>884</v>
+        <v>890</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>885</v>
+        <v>891</v>
       </c>
       <c r="D32" s="4" t="s">
         <v>487</v>
@@ -6822,13 +6881,13 @@
         <v>50</v>
       </c>
       <c r="F32" s="4" t="s">
-        <v>821</v>
+        <v>827</v>
       </c>
       <c r="G32" s="4" t="s">
         <v>35</v>
       </c>
       <c r="H32" s="4" t="s">
-        <v>822</v>
+        <v>828</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.25">
@@ -6836,10 +6895,10 @@
         <v>307</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>886</v>
+        <v>892</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>831</v>
+        <v>837</v>
       </c>
       <c r="D33" s="4" t="s">
         <v>269</v>
@@ -6848,10 +6907,10 @@
         <v>50</v>
       </c>
       <c r="F33" s="4" t="s">
-        <v>826</v>
+        <v>832</v>
       </c>
       <c r="G33" s="4" t="s">
-        <v>831</v>
+        <v>837</v>
       </c>
       <c r="H33" s="4" t="s">
         <v>35</v>
@@ -6862,10 +6921,10 @@
         <v>307</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>887</v>
+        <v>893</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>826</v>
+        <v>832</v>
       </c>
       <c r="D34" s="4" t="s">
         <v>269</v>
@@ -6874,7 +6933,7 @@
         <v>50</v>
       </c>
       <c r="F34" s="4" t="s">
-        <v>826</v>
+        <v>832</v>
       </c>
       <c r="G34" s="4" t="s">
         <v>35</v>
@@ -6888,10 +6947,10 @@
         <v>307</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>888</v>
+        <v>894</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>889</v>
+        <v>895</v>
       </c>
       <c r="D35" s="4" t="s">
         <v>269</v>
@@ -6900,7 +6959,7 @@
         <v>50</v>
       </c>
       <c r="F35" s="4" t="s">
-        <v>826</v>
+        <v>832</v>
       </c>
       <c r="G35" s="4" t="s">
         <v>35</v>
@@ -6911,7 +6970,7 @@
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A37" s="4" t="s">
-        <v>890</v>
+        <v>896</v>
       </c>
     </row>
   </sheetData>
@@ -6950,36 +7009,36 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>816</v>
+        <v>822</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>891</v>
+        <v>897</v>
       </c>
       <c r="C1" s="6" t="s">
         <v>58</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>892</v>
+        <v>898</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>893</v>
+        <v>899</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>894</v>
+        <v>900</v>
       </c>
       <c r="G1" s="6" t="s">
-        <v>895</v>
+        <v>901</v>
       </c>
       <c r="H1" s="6" t="s">
         <v>100</v>
       </c>
       <c r="I1" s="6" t="s">
-        <v>896</v>
+        <v>902</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>897</v>
+        <v>903</v>
       </c>
     </row>
   </sheetData>
@@ -6990,7 +7049,7 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D81"/>
+  <dimension ref="A1:D83"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="44" customWidth="1"/>
@@ -7001,12 +7060,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>898</v>
+        <v>904</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
-        <v>899</v>
+        <v>905</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -7035,7 +7094,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>900</v>
+        <v>906</v>
       </c>
       <c r="B7" s="4" t="s">
         <v>12</v>
@@ -7043,39 +7102,39 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>901</v>
+        <v>907</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>902</v>
+        <v>908</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>903</v>
+        <v>909</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>904</v>
+        <v>910</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>905</v>
+        <v>911</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>906</v>
+        <v>912</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>907</v>
+        <v>913</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>908</v>
+        <v>914</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
-        <v>909</v>
+        <v>915</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
@@ -7083,7 +7142,7 @@
         <v>110</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>910</v>
+        <v>916</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
@@ -7091,7 +7150,7 @@
         <v>110</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>911</v>
+        <v>917</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
@@ -7099,7 +7158,7 @@
         <v>110</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>912</v>
+        <v>918</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
@@ -7107,12 +7166,12 @@
         <v>110</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>913</v>
+        <v>919</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
-        <v>914</v>
+        <v>920</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
@@ -7123,178 +7182,178 @@
         <v>480</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>915</v>
+        <v>921</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>916</v>
+        <v>922</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="4" t="s">
-        <v>917</v>
+        <v>923</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>918</v>
+        <v>924</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>919</v>
+        <v>925</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>920</v>
+        <v>926</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="4" t="s">
-        <v>921</v>
+        <v>927</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>922</v>
+        <v>928</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>923</v>
+        <v>929</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>924</v>
+        <v>930</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="4" t="s">
-        <v>925</v>
+        <v>931</v>
       </c>
       <c r="B23" s="3" t="s">
+        <v>932</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>933</v>
+      </c>
+      <c r="D23" s="4" t="s">
         <v>926</v>
-      </c>
-      <c r="C23" s="4" t="s">
-        <v>927</v>
-      </c>
-      <c r="D23" s="4" t="s">
-        <v>920</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="4" t="s">
-        <v>928</v>
+        <v>934</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>929</v>
+        <v>935</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>927</v>
+        <v>933</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>924</v>
+        <v>930</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
+        <v>936</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>937</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>938</v>
+      </c>
+      <c r="D25" s="4" t="s">
         <v>930</v>
-      </c>
-      <c r="B25" s="3" t="s">
-        <v>931</v>
-      </c>
-      <c r="C25" s="4" t="s">
-        <v>932</v>
-      </c>
-      <c r="D25" s="4" t="s">
-        <v>924</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="4" t="s">
+        <v>939</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>940</v>
+      </c>
+      <c r="C26" s="4" t="s">
         <v>933</v>
       </c>
-      <c r="B26" s="3" t="s">
-        <v>934</v>
-      </c>
-      <c r="C26" s="4" t="s">
-        <v>927</v>
-      </c>
       <c r="D26" s="4" t="s">
-        <v>924</v>
+        <v>930</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="4" t="s">
-        <v>935</v>
+        <v>941</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>936</v>
+        <v>942</v>
       </c>
       <c r="C27" s="4" t="s">
         <v>119</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>937</v>
+        <v>943</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
-        <v>938</v>
+        <v>944</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>939</v>
+        <v>945</v>
       </c>
       <c r="C28" s="4" t="s">
         <v>600</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>924</v>
+        <v>930</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="4" t="s">
-        <v>940</v>
+        <v>946</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>941</v>
+        <v>947</v>
       </c>
       <c r="C29" s="4" t="s">
         <v>119</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>924</v>
+        <v>930</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="4" t="s">
-        <v>942</v>
+        <v>948</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>943</v>
+        <v>949</v>
       </c>
       <c r="C30" s="4" t="s">
         <v>611</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>920</v>
+        <v>926</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="4" t="s">
-        <v>944</v>
+        <v>950</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>945</v>
+        <v>951</v>
       </c>
       <c r="C31" s="4" t="s">
         <v>611</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>937</v>
+        <v>943</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="4" t="s">
-        <v>946</v>
+        <v>952</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>947</v>
+        <v>953</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>948</v>
+        <v>954</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>924</v>
+        <v>930</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
@@ -7302,13 +7361,13 @@
         <v>544</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>949</v>
+        <v>955</v>
       </c>
       <c r="C33" s="4" t="s">
         <v>611</v>
       </c>
       <c r="D33" s="4" t="s">
-        <v>937</v>
+        <v>943</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
@@ -7316,13 +7375,13 @@
         <v>541</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>950</v>
+        <v>956</v>
       </c>
       <c r="C34" s="4" t="s">
         <v>611</v>
       </c>
       <c r="D34" s="4" t="s">
-        <v>924</v>
+        <v>930</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
@@ -7336,7 +7395,7 @@
         <v>607</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>937</v>
+        <v>943</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
@@ -7350,7 +7409,7 @@
         <v>607</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>937</v>
+        <v>943</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
@@ -7364,7 +7423,7 @@
         <v>607</v>
       </c>
       <c r="D37" s="4" t="s">
-        <v>937</v>
+        <v>943</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
@@ -7378,7 +7437,7 @@
         <v>607</v>
       </c>
       <c r="D38" s="4" t="s">
-        <v>937</v>
+        <v>943</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
@@ -7392,7 +7451,7 @@
         <v>607</v>
       </c>
       <c r="D39" s="4" t="s">
-        <v>937</v>
+        <v>943</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
@@ -7406,7 +7465,7 @@
         <v>607</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>937</v>
+        <v>943</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
@@ -7420,12 +7479,12 @@
         <v>607</v>
       </c>
       <c r="D41" s="4" t="s">
-        <v>937</v>
+        <v>943</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42" s="4" t="s">
-        <v>951</v>
+        <v>957</v>
       </c>
       <c r="B42" s="3" t="s">
         <v>509</v>
@@ -7434,7 +7493,7 @@
         <v>607</v>
       </c>
       <c r="D42" s="4" t="s">
-        <v>920</v>
+        <v>926</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
@@ -7442,13 +7501,13 @@
         <v>31</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>952</v>
+        <v>958</v>
       </c>
       <c r="C43" s="4" t="s">
         <v>607</v>
       </c>
       <c r="D43" s="4" t="s">
-        <v>937</v>
+        <v>943</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
@@ -7462,7 +7521,7 @@
         <v>611</v>
       </c>
       <c r="D44" s="4" t="s">
-        <v>937</v>
+        <v>943</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
@@ -7476,7 +7535,7 @@
         <v>611</v>
       </c>
       <c r="D45" s="4" t="s">
-        <v>937</v>
+        <v>943</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
@@ -7490,7 +7549,7 @@
         <v>611</v>
       </c>
       <c r="D46" s="4" t="s">
-        <v>937</v>
+        <v>943</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
@@ -7504,7 +7563,7 @@
         <v>611</v>
       </c>
       <c r="D47" s="4" t="s">
-        <v>937</v>
+        <v>943</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
@@ -7518,7 +7577,7 @@
         <v>611</v>
       </c>
       <c r="D48" s="4" t="s">
-        <v>937</v>
+        <v>943</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
@@ -7532,7 +7591,7 @@
         <v>611</v>
       </c>
       <c r="D49" s="4" t="s">
-        <v>920</v>
+        <v>926</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
@@ -7546,7 +7605,7 @@
         <v>611</v>
       </c>
       <c r="D50" s="4" t="s">
-        <v>937</v>
+        <v>943</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
@@ -7560,7 +7619,7 @@
         <v>611</v>
       </c>
       <c r="D51" s="4" t="s">
-        <v>920</v>
+        <v>926</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
@@ -7574,7 +7633,7 @@
         <v>611</v>
       </c>
       <c r="D52" s="4" t="s">
-        <v>937</v>
+        <v>943</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
@@ -7582,27 +7641,27 @@
         <v>544</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>953</v>
+        <v>959</v>
       </c>
       <c r="C53" s="4" t="s">
         <v>611</v>
       </c>
       <c r="D53" s="4" t="s">
-        <v>937</v>
+        <v>943</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54" s="3" t="s">
-        <v>954</v>
+        <v>960</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>955</v>
+        <v>961</v>
       </c>
       <c r="C54" s="4" t="s">
         <v>611</v>
       </c>
       <c r="D54" s="4" t="s">
-        <v>924</v>
+        <v>930</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
@@ -7616,49 +7675,49 @@
         <v>611</v>
       </c>
       <c r="D55" s="4" t="s">
-        <v>937</v>
+        <v>943</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" s="4" t="s">
-        <v>956</v>
+        <v>962</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>957</v>
+        <v>963</v>
       </c>
       <c r="C56" s="4" t="s">
         <v>611</v>
       </c>
       <c r="D56" s="4" t="s">
-        <v>937</v>
+        <v>943</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57" s="4" t="s">
-        <v>958</v>
+        <v>964</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>959</v>
+        <v>965</v>
       </c>
       <c r="C57" s="4" t="s">
         <v>611</v>
       </c>
       <c r="D57" s="4" t="s">
-        <v>937</v>
+        <v>943</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58" s="4" t="s">
-        <v>960</v>
+        <v>966</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>961</v>
+        <v>967</v>
       </c>
       <c r="C58" s="4" t="s">
         <v>255</v>
       </c>
       <c r="D58" s="4" t="s">
-        <v>937</v>
+        <v>943</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
@@ -7666,13 +7725,13 @@
         <v>41</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>962</v>
+        <v>968</v>
       </c>
       <c r="C59" s="4" t="s">
         <v>166</v>
       </c>
       <c r="D59" s="4" t="s">
-        <v>937</v>
+        <v>943</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
@@ -7680,116 +7739,116 @@
         <v>42</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>963</v>
+        <v>969</v>
       </c>
       <c r="C60" s="4" t="s">
         <v>166</v>
       </c>
       <c r="D60" s="4" t="s">
-        <v>924</v>
+        <v>930</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61" s="4" t="s">
-        <v>964</v>
+        <v>970</v>
       </c>
       <c r="B61" s="3" t="s">
-        <v>965</v>
+        <v>971</v>
       </c>
       <c r="C61" s="4" t="s">
         <v>607</v>
       </c>
       <c r="D61" s="4" t="s">
-        <v>924</v>
+        <v>930</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62" s="4" t="s">
-        <v>966</v>
+        <v>972</v>
       </c>
       <c r="B62" s="3" t="s">
-        <v>967</v>
+        <v>973</v>
       </c>
       <c r="C62" s="4" t="s">
         <v>255</v>
       </c>
       <c r="D62" s="4" t="s">
-        <v>924</v>
+        <v>930</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A63" s="4" t="s">
-        <v>968</v>
+        <v>974</v>
       </c>
       <c r="B63" s="3" t="s">
-        <v>969</v>
+        <v>975</v>
       </c>
       <c r="C63" s="4" t="s">
         <v>607</v>
       </c>
       <c r="D63" s="4" t="s">
-        <v>937</v>
+        <v>943</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" s="4" t="s">
-        <v>970</v>
+        <v>976</v>
       </c>
       <c r="B64" s="3" t="s">
-        <v>971</v>
+        <v>977</v>
       </c>
       <c r="C64" s="4" t="s">
         <v>607</v>
       </c>
       <c r="D64" s="4" t="s">
-        <v>924</v>
+        <v>930</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A65" s="4" t="s">
-        <v>972</v>
+        <v>978</v>
       </c>
       <c r="B65" s="3" t="s">
-        <v>973</v>
+        <v>979</v>
       </c>
       <c r="C65" s="4" t="s">
         <v>607</v>
       </c>
       <c r="D65" s="4" t="s">
-        <v>920</v>
+        <v>926</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A66" s="4" t="s">
-        <v>974</v>
+        <v>980</v>
       </c>
       <c r="B66" s="3" t="s">
-        <v>975</v>
+        <v>981</v>
       </c>
       <c r="C66" s="4" t="s">
         <v>607</v>
       </c>
       <c r="D66" s="4" t="s">
-        <v>924</v>
+        <v>930</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A67" s="4" t="s">
-        <v>976</v>
+        <v>982</v>
       </c>
       <c r="B67" s="3" t="s">
-        <v>977</v>
+        <v>983</v>
       </c>
       <c r="C67" s="4" t="s">
         <v>598</v>
       </c>
       <c r="D67" s="4" t="s">
-        <v>924</v>
+        <v>930</v>
       </c>
     </row>
     <row r="69" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A69" s="5" t="s">
-        <v>978</v>
+        <v>984</v>
       </c>
     </row>
     <row r="70" spans="1:2" x14ac:dyDescent="0.25">
@@ -7797,7 +7856,7 @@
         <v>110</v>
       </c>
       <c r="B70" s="3" t="s">
-        <v>979</v>
+        <v>985</v>
       </c>
     </row>
     <row r="71" spans="1:2" x14ac:dyDescent="0.25">
@@ -7805,7 +7864,7 @@
         <v>110</v>
       </c>
       <c r="B71" s="3" t="s">
-        <v>980</v>
+        <v>986</v>
       </c>
     </row>
     <row r="72" spans="1:2" x14ac:dyDescent="0.25">
@@ -7813,7 +7872,7 @@
         <v>110</v>
       </c>
       <c r="B72" s="3" t="s">
-        <v>981</v>
+        <v>987</v>
       </c>
     </row>
     <row r="73" spans="1:2" x14ac:dyDescent="0.25">
@@ -7821,7 +7880,7 @@
         <v>110</v>
       </c>
       <c r="B73" s="3" t="s">
-        <v>982</v>
+        <v>988</v>
       </c>
     </row>
     <row r="74" spans="1:2" x14ac:dyDescent="0.25">
@@ -7829,7 +7888,7 @@
         <v>110</v>
       </c>
       <c r="B74" s="3" t="s">
-        <v>983</v>
+        <v>989</v>
       </c>
     </row>
     <row r="75" spans="1:2" x14ac:dyDescent="0.25">
@@ -7837,7 +7896,7 @@
         <v>110</v>
       </c>
       <c r="B75" s="3" t="s">
-        <v>984</v>
+        <v>990</v>
       </c>
     </row>
     <row r="76" spans="1:2" x14ac:dyDescent="0.25">
@@ -7845,7 +7904,7 @@
         <v>110</v>
       </c>
       <c r="B76" s="3" t="s">
-        <v>985</v>
+        <v>991</v>
       </c>
     </row>
     <row r="77" spans="1:2" x14ac:dyDescent="0.25">
@@ -7853,7 +7912,7 @@
         <v>110</v>
       </c>
       <c r="B77" s="3" t="s">
-        <v>986</v>
+        <v>992</v>
       </c>
     </row>
     <row r="78" spans="1:2" x14ac:dyDescent="0.25">
@@ -7861,7 +7920,7 @@
         <v>110</v>
       </c>
       <c r="B78" s="3" t="s">
-        <v>987</v>
+        <v>993</v>
       </c>
     </row>
     <row r="79" spans="1:2" x14ac:dyDescent="0.25">
@@ -7869,11 +7928,27 @@
         <v>110</v>
       </c>
       <c r="B79" s="3" t="s">
-        <v>988</v>
-      </c>
-    </row>
-    <row r="81" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A81" s="15" t="s">
+        <v>994</v>
+      </c>
+    </row>
+    <row r="80" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A80" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="B80" s="3" t="s">
+        <v>995</v>
+      </c>
+    </row>
+    <row r="81" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A81" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="B81" s="3" t="s">
+        <v>996</v>
+      </c>
+    </row>
+    <row r="83" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A83" s="15" t="s">
         <v>96</v>
       </c>
     </row>
@@ -15520,7 +15595,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:C21"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
@@ -15653,87 +15728,109 @@
         <v>627</v>
       </c>
       <c r="B12" s="4">
-        <v>6</v>
+        <v>106</v>
       </c>
       <c r="C12" s="4">
-        <v>6</v>
+        <v>106</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" s="4" t="s">
+      <c r="A13" s="3" t="s">
         <v>628</v>
       </c>
-      <c r="B13" s="4">
-        <v>77.5</v>
-      </c>
-      <c r="C13" s="4">
-        <v>77.5</v>
+      <c r="B13" s="4" t="s">
+        <v>629</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>629</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
-        <v>629</v>
+        <v>630</v>
       </c>
       <c r="B14" s="4">
-        <v>98.1</v>
+        <v>6</v>
       </c>
       <c r="C14" s="4">
-        <v>98.1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
-        <v>630</v>
-      </c>
-      <c r="B15" s="4" t="s">
         <v>631</v>
       </c>
-      <c r="C15" s="4" t="s">
-        <v>631</v>
+      <c r="B15" s="4">
+        <v>77.5</v>
+      </c>
+      <c r="C15" s="4">
+        <v>77.5</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
         <v>632</v>
       </c>
-      <c r="B16" s="4" t="s">
-        <v>633</v>
-      </c>
-      <c r="C16" s="4" t="s">
-        <v>633</v>
+      <c r="B16" s="4">
+        <v>98.1</v>
+      </c>
+      <c r="C16" s="4">
+        <v>98.1</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
+        <v>633</v>
+      </c>
+      <c r="B17" s="4" t="s">
         <v>634</v>
       </c>
-      <c r="B17" s="4" t="s">
-        <v>635</v>
-      </c>
       <c r="C17" s="4" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
+        <v>635</v>
+      </c>
+      <c r="B18" s="4" t="s">
         <v>636</v>
       </c>
-      <c r="B18" s="4">
-        <v>1</v>
-      </c>
-      <c r="C18" s="4">
-        <v>1</v>
+      <c r="C18" s="4" t="s">
+        <v>636</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
+        <v>637</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>638</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>638</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" s="4" t="s">
+        <v>639</v>
+      </c>
+      <c r="B20" s="4">
+        <v>1</v>
+      </c>
+      <c r="C20" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B19" s="4" t="s">
-        <v>637</v>
-      </c>
-      <c r="C19" s="4" t="s">
-        <v>637</v>
+      <c r="B21" s="4" t="s">
+        <v>640</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>640</v>
       </c>
     </row>
   </sheetData>

</xml_diff>